<commit_message>
Updated JPN_grids model - 2025-09-13 10:43
</commit_message>
<xml_diff>
--- a/VerveStacks_JPN_grids/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_JPN_grids/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_JPN_grids\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{18A5B0B5-FE8B-4060-9268-AE9895F60F3D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{203938AA-C9D6-4019-89EA-E7D2CE6B2A35}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -8465,7 +8465,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DE96781D-FF40-441B-82B2-DDD08DD456A8}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{811CF0A0-40D7-4938-A553-0772589F71F8}">
   <dimension ref="B9:D1116"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -20657,7 +20657,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{39994794-2E14-4EDD-A8E5-05C289883757}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7D6ECB70-EAC4-40C2-B31C-BE3002D47205}">
   <dimension ref="B9:H1116"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated JPN_grids model - 2025-09-13 11:56
</commit_message>
<xml_diff>
--- a/VerveStacks_JPN_grids/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_JPN_grids/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_JPN_grids\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{203938AA-C9D6-4019-89EA-E7D2CE6B2A35}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{52F587FF-CA44-4AC6-B8BA-1CD63B09155D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -8465,7 +8465,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{811CF0A0-40D7-4938-A553-0772589F71F8}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{930E3F8C-43F6-408F-85A3-54A628E6A6DE}">
   <dimension ref="B9:D1116"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -20657,7 +20657,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7D6ECB70-EAC4-40C2-B31C-BE3002D47205}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D87EE4CD-2117-435A-BBA1-E13663B369AB}">
   <dimension ref="B9:H1116"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated JPN_grids model - 2025-09-13 14:16
</commit_message>
<xml_diff>
--- a/VerveStacks_JPN_grids/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_JPN_grids/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_JPN_grids\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{52F587FF-CA44-4AC6-B8BA-1CD63B09155D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{4C2D6A8B-A5B7-49E3-A4D4-8D52EA0F14F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -8465,7 +8465,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{930E3F8C-43F6-408F-85A3-54A628E6A6DE}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{84929580-C975-4756-BFD0-BFE76589A487}">
   <dimension ref="B9:D1116"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -20657,7 +20657,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D87EE4CD-2117-435A-BBA1-E13663B369AB}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9CA0090C-C442-427F-AEB3-89A752407D9A}">
   <dimension ref="B9:H1116"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated JPN_grids model - 2025-09-13 15:02
</commit_message>
<xml_diff>
--- a/VerveStacks_JPN_grids/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_JPN_grids/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_JPN_grids\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{4C2D6A8B-A5B7-49E3-A4D4-8D52EA0F14F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{BFCD3FC7-B573-4DB1-8D9E-8DB096865B9A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -8465,7 +8465,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{84929580-C975-4756-BFD0-BFE76589A487}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B354EC7B-C474-4D19-8851-2C1628FA2EA5}">
   <dimension ref="B9:D1116"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -20657,7 +20657,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9CA0090C-C442-427F-AEB3-89A752407D9A}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{947A2A52-81AD-43F0-8033-E31053556CD3}">
   <dimension ref="B9:H1116"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated JPN_grids model - 2025-09-13 15:34
</commit_message>
<xml_diff>
--- a/VerveStacks_JPN_grids/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_JPN_grids/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_JPN_grids\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{BFCD3FC7-B573-4DB1-8D9E-8DB096865B9A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{404D212B-F7D4-4961-AA46-B37E7084EE8E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -8465,7 +8465,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B354EC7B-C474-4D19-8851-2C1628FA2EA5}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DBFC2BF2-FE72-42A7-9DC1-5135D47C259B}">
   <dimension ref="B9:D1116"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -20657,7 +20657,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{947A2A52-81AD-43F0-8033-E31053556CD3}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7017DECA-2082-4307-AE55-22DF3A8EED61}">
   <dimension ref="B9:H1116"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated JPN_grids model - 2025-09-13 16:09
</commit_message>
<xml_diff>
--- a/VerveStacks_JPN_grids/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_JPN_grids/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_JPN_grids\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{404D212B-F7D4-4961-AA46-B37E7084EE8E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{DE495724-AC9A-4D43-A2EB-7EA68D5B0459}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -8465,7 +8465,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DBFC2BF2-FE72-42A7-9DC1-5135D47C259B}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5748BDAD-89B7-4FBD-B1C8-9E30977DBA0D}">
   <dimension ref="B9:D1116"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -20657,7 +20657,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7017DECA-2082-4307-AE55-22DF3A8EED61}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{977D989B-FCC9-478A-98EF-178EAF52D7BA}">
   <dimension ref="B9:H1116"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated JPN_grids model - 2025-09-13 17:43
</commit_message>
<xml_diff>
--- a/VerveStacks_JPN_grids/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_JPN_grids/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_JPN_grids\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{DE495724-AC9A-4D43-A2EB-7EA68D5B0459}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{E8EE7BD8-FA47-40D1-AA49-B69E6978A866}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -8465,7 +8465,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5748BDAD-89B7-4FBD-B1C8-9E30977DBA0D}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F4E5EF1A-9B5C-4872-8BE6-5B72170025CB}">
   <dimension ref="B9:D1116"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -20657,7 +20657,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{977D989B-FCC9-478A-98EF-178EAF52D7BA}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F46C9979-19BF-44EE-93B4-7F6D8FF305D3}">
   <dimension ref="B9:H1116"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated JPN_grids model - 2025-09-14 19:43
</commit_message>
<xml_diff>
--- a/VerveStacks_JPN_grids/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_JPN_grids/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_JPN_grids\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E8EE7BD8-FA47-40D1-AA49-B69E6978A866}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{599233D9-AF68-4836-B27B-FF2AB355E1B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -8465,7 +8465,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F4E5EF1A-9B5C-4872-8BE6-5B72170025CB}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{52DE684E-139E-4C55-B5E8-1B2A36794B87}">
   <dimension ref="B9:D1116"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -20657,7 +20657,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F46C9979-19BF-44EE-93B4-7F6D8FF305D3}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{54503564-3A7D-450D-9A9B-5B5E477882AB}">
   <dimension ref="B9:H1116"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated JPN_grids model - 2025-09-15 01:04
</commit_message>
<xml_diff>
--- a/VerveStacks_JPN_grids/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_JPN_grids/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_JPN_grids\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{599233D9-AF68-4836-B27B-FF2AB355E1B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{1210BA40-CDFD-4C8F-9385-5E7A9BAED2EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1241,13 +1241,13 @@
     <t>g64</t>
   </si>
   <si>
-    <t>f97p50</t>
-  </si>
-  <si>
     <t>f96p10</t>
   </si>
   <si>
     <t>f96p90</t>
+  </si>
+  <si>
+    <t>f96p50</t>
   </si>
   <si>
     <t>grid_node</t>
@@ -8465,7 +8465,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{52DE684E-139E-4C55-B5E8-1B2A36794B87}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F10BE571-86D0-4FFB-B701-5D44FDB5B5EE}">
   <dimension ref="B9:D1116"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -20657,7 +20657,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{54503564-3A7D-450D-9A9B-5B5E477882AB}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6B4227E2-00F8-4928-B080-24E622175B97}">
   <dimension ref="B9:H1116"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -43248,7 +43248,7 @@
         <v>337</v>
       </c>
       <c r="U12" t="s">
-        <v>385</v>
+        <v>387</v>
       </c>
     </row>
     <row r="13" spans="2:24">
@@ -43291,7 +43291,7 @@
         <v>343</v>
       </c>
       <c r="U13" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
     </row>
     <row r="14" spans="2:24">
@@ -43334,7 +43334,7 @@
         <v>349</v>
       </c>
       <c r="U14" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
     </row>
     <row r="15" spans="2:24">
@@ -44151,11 +44151,11 @@
       </c>
       <c r="C36" t="str">
         <f t="shared" si="5"/>
-        <v>e 1.5 deg no OS.f97p50</v>
+        <v>e 1.5 deg no OS.f96p50</v>
       </c>
       <c r="H36" t="str">
         <f t="shared" si="2"/>
-        <v>e 1.5 deg no OS.f97p50</v>
+        <v>e 1.5 deg no OS.f96p50</v>
       </c>
       <c r="I36" t="str">
         <f t="shared" si="3"/>
@@ -44163,7 +44163,7 @@
       </c>
       <c r="J36" t="str">
         <f t="shared" si="4"/>
-        <v>f97p50</v>
+        <v>f96p50</v>
       </c>
       <c r="N36">
         <v>5</v>
@@ -44188,11 +44188,11 @@
       </c>
       <c r="C37" t="str">
         <f t="shared" si="5"/>
-        <v>d 1.5 deg OS.f97p50</v>
+        <v>d 1.5 deg OS.f96p50</v>
       </c>
       <c r="H37" t="str">
         <f t="shared" si="2"/>
-        <v>d 1.5 deg OS.f97p50</v>
+        <v>d 1.5 deg OS.f96p50</v>
       </c>
       <c r="I37" t="str">
         <f t="shared" si="3"/>
@@ -44200,7 +44200,7 @@
       </c>
       <c r="J37" t="str">
         <f t="shared" si="4"/>
-        <v>f97p50</v>
+        <v>f96p50</v>
       </c>
       <c r="N37">
         <v>5</v>
@@ -44225,11 +44225,11 @@
       </c>
       <c r="C38" t="str">
         <f t="shared" si="5"/>
-        <v>c 2 deg (67%).f97p50</v>
+        <v>c 2 deg (67%).f96p50</v>
       </c>
       <c r="H38" t="str">
         <f t="shared" si="2"/>
-        <v>c 2 deg (67%).f97p50</v>
+        <v>c 2 deg (67%).f96p50</v>
       </c>
       <c r="I38" t="str">
         <f t="shared" si="3"/>
@@ -44237,7 +44237,7 @@
       </c>
       <c r="J38" t="str">
         <f t="shared" si="4"/>
-        <v>f97p50</v>
+        <v>f96p50</v>
       </c>
       <c r="N38">
         <v>5</v>
@@ -44262,11 +44262,11 @@
       </c>
       <c r="C39" t="str">
         <f t="shared" si="5"/>
-        <v>b 2 deg (50%).f97p50</v>
+        <v>b 2 deg (50%).f96p50</v>
       </c>
       <c r="H39" t="str">
         <f t="shared" si="2"/>
-        <v>b 2 deg (50%).f97p50</v>
+        <v>b 2 deg (50%).f96p50</v>
       </c>
       <c r="I39" t="str">
         <f t="shared" si="3"/>
@@ -44274,7 +44274,7 @@
       </c>
       <c r="J39" t="str">
         <f t="shared" si="4"/>
-        <v>f97p50</v>
+        <v>f96p50</v>
       </c>
       <c r="N39">
         <v>5</v>
@@ -44299,11 +44299,11 @@
       </c>
       <c r="C40" t="str">
         <f t="shared" si="5"/>
-        <v>a 3 deg.f97p50</v>
+        <v>a 3 deg.f96p50</v>
       </c>
       <c r="H40" t="str">
         <f t="shared" si="2"/>
-        <v>a 3 deg.f97p50</v>
+        <v>a 3 deg.f96p50</v>
       </c>
       <c r="I40" t="str">
         <f t="shared" si="3"/>
@@ -44311,7 +44311,7 @@
       </c>
       <c r="J40" t="str">
         <f t="shared" si="4"/>
-        <v>f97p50</v>
+        <v>f96p50</v>
       </c>
       <c r="N40">
         <v>5</v>

</xml_diff>

<commit_message>
Updated JPN_grids model - 2025-09-17 02:43
</commit_message>
<xml_diff>
--- a/VerveStacks_JPN_grids/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_JPN_grids/ReportDefs_vervestacks.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_JPN_grids\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{1210BA40-CDFD-4C8F-9385-5E7A9BAED2EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{637937DE-252C-49C4-A4CF-8AE3ABFF36C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="735" yWindow="735" windowWidth="21600" windowHeight="12682" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ScenMap_OLD" sheetId="70" r:id="rId1"/>
@@ -8465,7 +8465,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F10BE571-86D0-4FFB-B701-5D44FDB5B5EE}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0509CF8E-53F2-4C0B-9059-B4326F3E6AAD}">
   <dimension ref="B9:D1116"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -20657,7 +20657,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6B4227E2-00F8-4928-B080-24E622175B97}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F7CD61AC-9DD2-453E-9229-E7CF0D9DC363}">
   <dimension ref="B9:H1116"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated JPN_grids model - 2025-09-19 11:38
</commit_message>
<xml_diff>
--- a/VerveStacks_JPN_grids/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_JPN_grids/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_JPN_grids\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{4C2779D2-3A95-44A2-B517-8CD1EA13045C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{F2D95EA3-3B8B-4F3F-95E2-662C74A67532}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -8891,7 +8891,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2C1FF46B-2796-47BF-B66F-B1045190FA08}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{61AB5D57-7AD9-425C-9AA1-FD46D9C6E852}">
   <dimension ref="B9:D298"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -12085,7 +12085,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5A71B8A6-7CFB-4AEA-81F7-C63D0F7F3BED}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0883FD8E-757D-4FAA-A07B-951893F66083}">
   <dimension ref="B9:H298"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated JPN_grids model - 2025-09-19 12:18
</commit_message>
<xml_diff>
--- a/VerveStacks_JPN_grids/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_JPN_grids/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_JPN_grids\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F2D95EA3-3B8B-4F3F-95E2-662C74A67532}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{74BA20FC-5413-47FB-AA60-189D02ABFCE9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -8891,7 +8891,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{61AB5D57-7AD9-425C-9AA1-FD46D9C6E852}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2DB8703E-96EB-46F4-A765-E9919C0F8F56}">
   <dimension ref="B9:D298"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -12085,7 +12085,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0883FD8E-757D-4FAA-A07B-951893F66083}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D439DC9C-53BB-4AD0-B66F-8E82670D1693}">
   <dimension ref="B9:H298"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated JPN_grids model - 2025-09-19 14:22
</commit_message>
<xml_diff>
--- a/VerveStacks_JPN_grids/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_JPN_grids/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_JPN_grids\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{74BA20FC-5413-47FB-AA60-189D02ABFCE9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{34DC773A-AEAB-4721-8DBA-0693691F6C06}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -8891,7 +8891,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2DB8703E-96EB-46F4-A765-E9919C0F8F56}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0EC46BFE-99A6-43F1-AE99-E27934AFC484}">
   <dimension ref="B9:D298"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -12085,7 +12085,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D439DC9C-53BB-4AD0-B66F-8E82670D1693}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0ABBA048-A8B6-4396-B3A8-A7CF91D711E3}">
   <dimension ref="B9:H298"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated JPN_grids model - 2025-09-19 22:30
</commit_message>
<xml_diff>
--- a/VerveStacks_JPN_grids/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_JPN_grids/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_JPN_grids\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{7AC33804-0D58-4679-8984-A8B21FE0E74B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{64DF6711-24B1-4A2A-A508-DFBE767D68FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -8891,7 +8891,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8220F6F9-C22B-458D-A490-3CA95DBFEE5E}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{39179948-8D39-4D3F-9A9A-F666D700FBF0}">
   <dimension ref="B9:D298"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -12085,7 +12085,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5E37C466-FEE5-47BD-A79F-F2CEBA3186BC}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{689A0A43-949E-47D9-8BC6-5C3E7DF09684}">
   <dimension ref="B9:H298"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated JPN_grids model - 2025-09-19 22:51
</commit_message>
<xml_diff>
--- a/VerveStacks_JPN_grids/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_JPN_grids/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_JPN_grids\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{64DF6711-24B1-4A2A-A508-DFBE767D68FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{09868DF0-E8C5-4B60-AE77-65F0DC4A3AC9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -8891,7 +8891,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{39179948-8D39-4D3F-9A9A-F666D700FBF0}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DF52B901-8A73-4297-9939-7C24A33E88DC}">
   <dimension ref="B9:D298"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -12085,7 +12085,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{689A0A43-949E-47D9-8BC6-5C3E7DF09684}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{68DEF76B-EE4C-4B44-ABA5-02D0D3E0F8AA}">
   <dimension ref="B9:H298"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated JPN_grids model - 2025-09-19 23:05
</commit_message>
<xml_diff>
--- a/VerveStacks_JPN_grids/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_JPN_grids/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_JPN_grids\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{09868DF0-E8C5-4B60-AE77-65F0DC4A3AC9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{AFF35090-E665-44C9-9C7C-A58F7CE71979}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -8891,7 +8891,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DF52B901-8A73-4297-9939-7C24A33E88DC}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D1BF1B6A-07C3-4AE8-91E2-1570C4BEE289}">
   <dimension ref="B9:D298"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -12085,7 +12085,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{68DEF76B-EE4C-4B44-ABA5-02D0D3E0F8AA}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{118B2726-F61C-4181-9ABD-719AEC63149E}">
   <dimension ref="B9:H298"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated JPN_grids model - 2025-09-20 09:04
</commit_message>
<xml_diff>
--- a/VerveStacks_JPN_grids/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_JPN_grids/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_JPN_grids\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{AFF35090-E665-44C9-9C7C-A58F7CE71979}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{FBED1195-F36F-4BCC-B1C2-D7C66758D91A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -8891,7 +8891,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D1BF1B6A-07C3-4AE8-91E2-1570C4BEE289}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FE11C847-FD89-4245-A8F8-178664313562}">
   <dimension ref="B9:D298"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -12085,7 +12085,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{118B2726-F61C-4181-9ABD-719AEC63149E}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B53FD76B-FB09-4255-9052-55474412E4EA}">
   <dimension ref="B9:H298"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated JPN_grids model - 2025-09-22 03:24
</commit_message>
<xml_diff>
--- a/VerveStacks_JPN_grids/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_JPN_grids/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_JPN_grids\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{38352A79-3268-41B7-8633-79A392964542}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{4AEBD19E-40D1-4F38-AF1C-E80959B29F8D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -84,7 +84,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2852" uniqueCount="744">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2852" uniqueCount="745">
   <si>
     <t>Unit</t>
   </si>
@@ -2298,6 +2298,9 @@
   </si>
   <si>
     <t>Hokkaidō</t>
+  </si>
+  <si>
+    <t>Yamagata</t>
   </si>
   <si>
     <t>Akita</t>
@@ -8906,24 +8909,24 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2186A339-34DA-49E4-BAB6-D7223F8F388F}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4BA644FC-647E-460B-886F-4CF924F99980}">
   <dimension ref="B9:D298"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
     <row r="9" spans="2:4">
       <c r="B9" t="s">
-        <v>740</v>
+        <v>741</v>
       </c>
     </row>
     <row r="10" spans="2:4">
       <c r="B10" t="s">
-        <v>741</v>
+        <v>742</v>
       </c>
       <c r="C10" t="s">
-        <v>742</v>
+        <v>743</v>
       </c>
       <c r="D10" t="s">
-        <v>743</v>
+        <v>744</v>
       </c>
     </row>
     <row r="11" spans="2:4">
@@ -10933,10 +10936,10 @@
         <v>587</v>
       </c>
       <c r="C193">
-        <v>41.3361912214217</v>
+        <v>27.229708944713892</v>
       </c>
       <c r="D193">
-        <v>140.82133755355883</v>
+        <v>128.34501674818958</v>
       </c>
     </row>
     <row r="194" spans="2:4">
@@ -10944,10 +10947,10 @@
         <v>588</v>
       </c>
       <c r="C194">
-        <v>40.045024127788608</v>
+        <v>24.81653263538637</v>
       </c>
       <c r="D194">
-        <v>140.08826559663316</v>
+        <v>124.47994184709124</v>
       </c>
     </row>
     <row r="195" spans="2:4">
@@ -10955,10 +10958,10 @@
         <v>589</v>
       </c>
       <c r="C195">
-        <v>42.76546822805534</v>
+        <v>25.790796362754623</v>
       </c>
       <c r="D195">
-        <v>142.3661927191954</v>
+        <v>138.21329309141947</v>
       </c>
     </row>
     <row r="196" spans="2:4">
@@ -10966,10 +10969,10 @@
         <v>590</v>
       </c>
       <c r="C196">
-        <v>42.492460260496109</v>
+        <v>33.659849545344365</v>
       </c>
       <c r="D196">
-        <v>140.46889911272919</v>
+        <v>129.68428282334222</v>
       </c>
     </row>
     <row r="197" spans="2:4">
@@ -10977,10 +10980,10 @@
         <v>591</v>
       </c>
       <c r="C197">
-        <v>44.41957532562013</v>
+        <v>30.737058363239601</v>
       </c>
       <c r="D197">
-        <v>141.45572674705218</v>
+        <v>130.61472030713247</v>
       </c>
     </row>
     <row r="198" spans="2:4">
@@ -10988,10 +10991,10 @@
         <v>592</v>
       </c>
       <c r="C198">
-        <v>44.390376612512185</v>
+        <v>32.431931356412775</v>
       </c>
       <c r="D198">
-        <v>142.60916164431279</v>
+        <v>130.39458183486042</v>
       </c>
     </row>
     <row r="199" spans="2:4">
@@ -10999,10 +11002,10 @@
         <v>593</v>
       </c>
       <c r="C199">
-        <v>43.969915143757859</v>
+        <v>31.546446690591694</v>
       </c>
       <c r="D199">
-        <v>144.34572196185522</v>
+        <v>131.40418241459082</v>
       </c>
     </row>
     <row r="200" spans="2:4">
@@ -11010,10 +11013,10 @@
         <v>594</v>
       </c>
       <c r="C200">
-        <v>43.147679382638273</v>
+        <v>33.276315860814783</v>
       </c>
       <c r="D200">
-        <v>145.02240376824813</v>
+        <v>132.4954976807833</v>
       </c>
     </row>
     <row r="201" spans="2:4">
@@ -11021,10 +11024,10 @@
         <v>595</v>
       </c>
       <c r="C201">
-        <v>42.877883273520922</v>
+        <v>33.8846796362755</v>
       </c>
       <c r="D201">
-        <v>143.64084508019593</v>
+        <v>135.62287055132165</v>
       </c>
     </row>
     <row r="202" spans="2:4">
@@ -11032,10 +11035,10 @@
         <v>596</v>
       </c>
       <c r="C202">
-        <v>33.659849545344365</v>
+        <v>35.233660181862305</v>
       </c>
       <c r="D202">
-        <v>129.68428282334222</v>
+        <v>137.47317236567724</v>
       </c>
     </row>
     <row r="203" spans="2:4">
@@ -11043,10 +11046,10 @@
         <v>597</v>
       </c>
       <c r="C203">
-        <v>30.737058363239601</v>
+        <v>35.183697939433166</v>
       </c>
       <c r="D203">
-        <v>130.61472030713247</v>
+        <v>135.11575079479454</v>
       </c>
     </row>
     <row r="204" spans="2:4">
@@ -11054,10 +11057,10 @@
         <v>598</v>
       </c>
       <c r="C204">
-        <v>32.431931356412775</v>
+        <v>34.424271854510224</v>
       </c>
       <c r="D204">
-        <v>130.39458183486042</v>
+        <v>133.6245445918176</v>
       </c>
     </row>
     <row r="205" spans="2:4">
@@ -11065,10 +11068,10 @@
         <v>599</v>
       </c>
       <c r="C205">
-        <v>35.233660181862305</v>
+        <v>34.887767734275947</v>
       </c>
       <c r="D205">
-        <v>137.47317236567724</v>
+        <v>132.33028219449398</v>
       </c>
     </row>
     <row r="206" spans="2:4">
@@ -11076,10 +11079,10 @@
         <v>600</v>
       </c>
       <c r="C206">
-        <v>34.484226545425187</v>
+        <v>43.969915143757859</v>
       </c>
       <c r="D206">
-        <v>135.60916461195606</v>
+        <v>144.34572196185522</v>
       </c>
     </row>
     <row r="207" spans="2:4">
@@ -11087,10 +11090,10 @@
         <v>601</v>
       </c>
       <c r="C207">
-        <v>31.546446690591694</v>
+        <v>43.147679382638273</v>
       </c>
       <c r="D207">
-        <v>131.40418241459082</v>
+        <v>145.02240376824813</v>
       </c>
     </row>
     <row r="208" spans="2:4">
@@ -11098,10 +11101,10 @@
         <v>602</v>
       </c>
       <c r="C208">
-        <v>33.276315860814783</v>
+        <v>42.877883273520922</v>
       </c>
       <c r="D208">
-        <v>132.4954976807833</v>
+        <v>143.64084508019593</v>
       </c>
     </row>
     <row r="209" spans="2:4">
@@ -11109,10 +11112,10 @@
         <v>603</v>
       </c>
       <c r="C209">
-        <v>35.49060885721218</v>
+        <v>44.41957532562013</v>
       </c>
       <c r="D209">
-        <v>133.84305642513195</v>
+        <v>141.45572674705218</v>
       </c>
     </row>
     <row r="210" spans="2:4">
@@ -11120,10 +11123,10 @@
         <v>604</v>
       </c>
       <c r="C210">
-        <v>34.334339818137771</v>
+        <v>44.390376612512185</v>
       </c>
       <c r="D210">
-        <v>131.79891346832002</v>
+        <v>142.60916164431279</v>
       </c>
     </row>
     <row r="211" spans="2:4">
@@ -11131,10 +11134,10 @@
         <v>605</v>
       </c>
       <c r="C211">
-        <v>34.424271854510224</v>
+        <v>42.76546822805534</v>
       </c>
       <c r="D211">
-        <v>133.6245445918176</v>
+        <v>142.3661927191954</v>
       </c>
     </row>
     <row r="212" spans="2:4">
@@ -11142,10 +11145,10 @@
         <v>606</v>
       </c>
       <c r="C212">
-        <v>28.263927362997119</v>
+        <v>42.492460260496109</v>
       </c>
       <c r="D212">
-        <v>129.33184438251254</v>
+        <v>140.46889911272919</v>
       </c>
     </row>
     <row r="213" spans="2:4">
@@ -11153,10 +11156,10 @@
         <v>607</v>
       </c>
       <c r="C213">
-        <v>26.853629519883636</v>
+        <v>34.896415045465609</v>
       </c>
       <c r="D213">
-        <v>127.98617033570848</v>
+        <v>139.44682763432323</v>
       </c>
     </row>
     <row r="214" spans="2:4">
@@ -11164,10 +11167,10 @@
         <v>608</v>
       </c>
       <c r="C214">
-        <v>24.81653263538637</v>
+        <v>37.931621273035937</v>
       </c>
       <c r="D214">
-        <v>124.47994184709124</v>
+        <v>141.09154035819489</v>
       </c>
     </row>
     <row r="215" spans="2:4">
@@ -11175,10 +11178,10 @@
         <v>609</v>
       </c>
       <c r="C215">
-        <v>25.790796362754623</v>
+        <v>36.357810636517982</v>
       </c>
       <c r="D215">
-        <v>138.21329309141947</v>
+        <v>140.55700872293659</v>
       </c>
     </row>
     <row r="216" spans="2:4">
@@ -11186,10 +11189,10 @@
         <v>610</v>
       </c>
       <c r="C216">
-        <v>34.896415045465609</v>
+        <v>36.492708691076665</v>
       </c>
       <c r="D216">
-        <v>139.44682763432323</v>
+        <v>139.29880348917476</v>
       </c>
     </row>
     <row r="217" spans="2:4">
@@ -11197,10 +11200,10 @@
         <v>611</v>
       </c>
       <c r="C217">
-        <v>36.357810636517982</v>
+        <v>36.651819216966402</v>
       </c>
       <c r="D217">
-        <v>140.55700872293659</v>
+        <v>137.30237527512134</v>
       </c>
     </row>
     <row r="218" spans="2:4">
@@ -11208,10 +11211,10 @@
         <v>612</v>
       </c>
       <c r="C218">
-        <v>36.492708691076665</v>
+        <v>37.831696788177652</v>
       </c>
       <c r="D218">
-        <v>139.29880348917476</v>
+        <v>138.0488218190323</v>
       </c>
     </row>
     <row r="219" spans="2:4">
@@ -11219,10 +11222,10 @@
         <v>613</v>
       </c>
       <c r="C219">
-        <v>39.834029734760925</v>
+        <v>38.066519327594612</v>
       </c>
       <c r="D219">
-        <v>141.47741526648781</v>
+        <v>139.79221730633628</v>
       </c>
     </row>
     <row r="220" spans="2:4">
@@ -11230,10 +11233,10 @@
         <v>614</v>
       </c>
       <c r="C220">
-        <v>38.156451363967072</v>
+        <v>39.376957571878961</v>
       </c>
       <c r="D220">
-        <v>140.92706908580772</v>
+        <v>141.38523905888621</v>
       </c>
     </row>
     <row r="221" spans="2:4">
@@ -11241,10 +11244,10 @@
         <v>615</v>
       </c>
       <c r="C221">
-        <v>38.060095610710867</v>
+        <v>39.955092091416148</v>
       </c>
       <c r="D221">
-        <v>139.23536456982546</v>
+        <v>139.94024145148472</v>
       </c>
     </row>
     <row r="222" spans="2:4">
@@ -11252,10 +11255,10 @@
         <v>616</v>
       </c>
       <c r="C222">
-        <v>37.63184781846109</v>
+        <v>40.449718291464649</v>
       </c>
       <c r="D222">
-        <v>136.89752291232216</v>
+        <v>141.07509323095616</v>
       </c>
     </row>
     <row r="223" spans="2:4">
@@ -11263,10 +11266,10 @@
         <v>617</v>
       </c>
       <c r="C223">
-        <v>36.651819216966402</v>
+        <v>41.3361912214217</v>
       </c>
       <c r="D223">
-        <v>137.30237527512134</v>
+        <v>140.82133755355883</v>
       </c>
     </row>
     <row r="224" spans="2:4">
@@ -11538,10 +11541,10 @@
         <v>642</v>
       </c>
       <c r="C248">
-        <v>42.806884297437385</v>
+        <v>42.668041855318521</v>
       </c>
       <c r="D248">
-        <v>141.06989940130185</v>
+        <v>141.20667024886589</v>
       </c>
     </row>
     <row r="249" spans="2:4">
@@ -11549,10 +11552,10 @@
         <v>643</v>
       </c>
       <c r="C249">
-        <v>41.817969987702703</v>
+        <v>42.153430758298363</v>
       </c>
       <c r="D249">
-        <v>140.68036217722695</v>
+        <v>140.65295029849574</v>
       </c>
     </row>
     <row r="250" spans="2:4">
@@ -11692,10 +11695,10 @@
         <v>656</v>
       </c>
       <c r="C262">
-        <v>31.550192137224879</v>
+        <v>33.380951449092692</v>
       </c>
       <c r="D262">
-        <v>131.70164591938115</v>
+        <v>133.88858020407105</v>
       </c>
     </row>
     <row r="263" spans="2:4">
@@ -11703,10 +11706,10 @@
         <v>657</v>
       </c>
       <c r="C263">
-        <v>33.006234630874133</v>
+        <v>31.550192137224879</v>
       </c>
       <c r="D263">
-        <v>134.62653033705877</v>
+        <v>131.70164591938115</v>
       </c>
     </row>
     <row r="264" spans="2:4">
@@ -11714,10 +11717,10 @@
         <v>658</v>
       </c>
       <c r="C264">
-        <v>33.380951449092692</v>
+        <v>33.006234630874133</v>
       </c>
       <c r="D264">
-        <v>133.88858020407105</v>
+        <v>134.62653033705877</v>
       </c>
     </row>
     <row r="265" spans="2:4">
@@ -11736,10 +11739,10 @@
         <v>660</v>
       </c>
       <c r="C266">
-        <v>31.935615150249681</v>
+        <v>32.060074664872275</v>
       </c>
       <c r="D266">
-        <v>129.11096992059461</v>
+        <v>129.14882070629113</v>
       </c>
     </row>
     <row r="267" spans="2:4">
@@ -11758,10 +11761,10 @@
         <v>662</v>
       </c>
       <c r="C268">
-        <v>33.409055210459087</v>
+        <v>33.477307202348889</v>
       </c>
       <c r="D268">
-        <v>128.79554670645661</v>
+        <v>128.707228206498</v>
       </c>
     </row>
     <row r="269" spans="2:4">
@@ -11769,10 +11772,10 @@
         <v>663</v>
       </c>
       <c r="C269">
-        <v>43.198532086418936</v>
+        <v>41.382257626347794</v>
       </c>
       <c r="D269">
-        <v>140.92789175632942</v>
+        <v>140.21980443639964</v>
       </c>
     </row>
     <row r="270" spans="2:4">
@@ -11780,10 +11783,10 @@
         <v>664</v>
       </c>
       <c r="C270">
-        <v>41.449853601398999</v>
+        <v>42.598985177269242</v>
       </c>
       <c r="D270">
-        <v>142.07930331134563</v>
+        <v>141.89612420032034</v>
       </c>
     </row>
     <row r="271" spans="2:4">
@@ -11791,10 +11794,10 @@
         <v>665</v>
       </c>
       <c r="C271">
-        <v>41.382257626347794</v>
+        <v>41.449853601398999</v>
       </c>
       <c r="D271">
-        <v>140.21980443639964</v>
+        <v>142.07930331134563</v>
       </c>
     </row>
     <row r="272" spans="2:4">
@@ -11802,10 +11805,10 @@
         <v>666</v>
       </c>
       <c r="C272">
-        <v>42.767607745467593</v>
+        <v>43.562542709831241</v>
       </c>
       <c r="D272">
-        <v>144.72231619899657</v>
+        <v>140.28115734393396</v>
       </c>
     </row>
     <row r="273" spans="2:4">
@@ -11813,10 +11816,10 @@
         <v>667</v>
       </c>
       <c r="C273">
-        <v>43.947965722856047</v>
+        <v>45.027150159325508</v>
       </c>
       <c r="D273">
-        <v>144.48680019910688</v>
+        <v>140.05909940118082</v>
       </c>
     </row>
     <row r="274" spans="2:4">
@@ -11824,10 +11827,10 @@
         <v>668</v>
       </c>
       <c r="C274">
-        <v>44.697399359293172</v>
+        <v>45.222002904799162</v>
       </c>
       <c r="D274">
-        <v>144.6438108657</v>
+        <v>141.73911353372725</v>
       </c>
     </row>
     <row r="275" spans="2:4">
@@ -11835,10 +11838,10 @@
         <v>669</v>
       </c>
       <c r="C275">
-        <v>44.62245599564946</v>
+        <v>42.767607745467593</v>
       </c>
       <c r="D275">
-        <v>140.22939558571642</v>
+        <v>144.72231619899657</v>
       </c>
     </row>
     <row r="276" spans="2:4">
@@ -11846,10 +11849,10 @@
         <v>670</v>
       </c>
       <c r="C276">
-        <v>45.521776359374002</v>
+        <v>43.947965722856047</v>
       </c>
       <c r="D276">
-        <v>141.89612420032034</v>
+        <v>144.48680019910688</v>
       </c>
     </row>
     <row r="277" spans="2:4">
@@ -11857,10 +11860,10 @@
         <v>671</v>
       </c>
       <c r="C277">
-        <v>44.959701132046163</v>
+        <v>44.697399359293172</v>
       </c>
       <c r="D277">
-        <v>143.19146219971361</v>
+        <v>144.6438108657</v>
       </c>
     </row>
     <row r="278" spans="2:4">
@@ -11868,10 +11871,10 @@
         <v>672</v>
       </c>
       <c r="C278">
-        <v>39.345561508501049</v>
+        <v>44.959701132046163</v>
       </c>
       <c r="D278">
-        <v>139.05607831929763</v>
+        <v>143.19146219971361</v>
       </c>
     </row>
     <row r="279" spans="2:4">
@@ -11879,10 +11882,10 @@
         <v>673</v>
       </c>
       <c r="C279">
-        <v>37.877553267715399</v>
+        <v>39.345561508501049</v>
       </c>
       <c r="D279">
-        <v>138.12786820208541</v>
+        <v>139.05607831929763</v>
       </c>
     </row>
     <row r="280" spans="2:4">
@@ -11890,10 +11893,10 @@
         <v>674</v>
       </c>
       <c r="C280">
-        <v>37.315478040387561</v>
+        <v>37.877553267715399</v>
       </c>
       <c r="D280">
-        <v>136.59701420280243</v>
+        <v>138.12786820208541</v>
       </c>
     </row>
     <row r="281" spans="2:4">
@@ -11901,10 +11904,10 @@
         <v>675</v>
       </c>
       <c r="C281">
-        <v>38.597009558695028</v>
+        <v>37.315478040387561</v>
       </c>
       <c r="D281">
-        <v>136.66766900276934</v>
+        <v>136.59701420280243</v>
       </c>
     </row>
     <row r="282" spans="2:4">
@@ -11912,10 +11915,10 @@
         <v>676</v>
       </c>
       <c r="C282">
-        <v>34.920172840852004</v>
+        <v>38.597009558695028</v>
       </c>
       <c r="D282">
-        <v>130.06597435970772</v>
+        <v>136.66766900276934</v>
       </c>
     </row>
     <row r="283" spans="2:4">
@@ -11923,10 +11926,10 @@
         <v>677</v>
       </c>
       <c r="C283">
-        <v>35.577368491266093</v>
+        <v>34.920172840852004</v>
       </c>
       <c r="D283">
-        <v>132.02256882032972</v>
+        <v>130.06597435970772</v>
       </c>
     </row>
     <row r="284" spans="2:4">
@@ -11934,10 +11937,10 @@
         <v>678</v>
       </c>
       <c r="C284">
-        <v>37.592768485869293</v>
+        <v>35.577368491266093</v>
       </c>
       <c r="D284">
-        <v>133.24483647103926</v>
+        <v>132.02256882032972</v>
       </c>
     </row>
     <row r="285" spans="2:4">
@@ -11945,10 +11948,10 @@
         <v>679</v>
       </c>
       <c r="C285">
-        <v>36.303742631197451</v>
+        <v>37.592768485869293</v>
       </c>
       <c r="D285">
-        <v>135.77270820318856</v>
+        <v>133.24483647103926</v>
       </c>
     </row>
     <row r="286" spans="2:4">
@@ -11956,10 +11959,10 @@
         <v>680</v>
       </c>
       <c r="C286">
-        <v>36.327408956558621</v>
+        <v>36.303742631197451</v>
       </c>
       <c r="D286">
-        <v>134.24805199337632</v>
+        <v>135.77270820318856</v>
       </c>
     </row>
     <row r="287" spans="2:4">
@@ -11967,10 +11970,10 @@
         <v>681</v>
       </c>
       <c r="C287">
-        <v>26.989353149764732</v>
+        <v>36.327408956558621</v>
       </c>
       <c r="D287">
-        <v>141.88490915270651</v>
+        <v>134.24805199337632</v>
       </c>
     </row>
     <row r="288" spans="2:4">
@@ -11978,10 +11981,10 @@
         <v>682</v>
       </c>
       <c r="C288">
-        <v>23.983053648171296</v>
+        <v>26.989353149764732</v>
       </c>
       <c r="D288">
-        <v>153.43640819491492</v>
+        <v>141.88490915270651</v>
       </c>
     </row>
     <row r="289" spans="2:4">
@@ -11989,10 +11992,10 @@
         <v>683</v>
       </c>
       <c r="C289">
-        <v>24.741052240453403</v>
+        <v>23.983053648171296</v>
       </c>
       <c r="D289">
-        <v>141.39144705769962</v>
+        <v>153.43640819491492</v>
       </c>
     </row>
     <row r="290" spans="2:4">
@@ -12000,10 +12003,10 @@
         <v>684</v>
       </c>
       <c r="C290">
-        <v>22.863899417758542</v>
+        <v>24.741052240453403</v>
       </c>
       <c r="D290">
-        <v>141.18957620065129</v>
+        <v>141.39144705769962</v>
       </c>
     </row>
     <row r="291" spans="2:4">
@@ -12011,10 +12014,10 @@
         <v>685</v>
       </c>
       <c r="C291">
-        <v>32.219329312615159</v>
+        <v>22.863899417758542</v>
       </c>
       <c r="D291">
-        <v>139.3839535348304</v>
+        <v>141.18957620065129</v>
       </c>
     </row>
     <row r="292" spans="2:4">
@@ -12022,10 +12025,10 @@
         <v>686</v>
       </c>
       <c r="C292">
-        <v>30.682990357919081</v>
+        <v>31.113914698870417</v>
       </c>
       <c r="D292">
-        <v>139.59984320139591</v>
+        <v>139.50171153477521</v>
       </c>
     </row>
     <row r="293" spans="2:4">
@@ -12033,10 +12036,10 @@
         <v>687</v>
       </c>
       <c r="C293">
-        <v>33.830611630954962</v>
+        <v>34.205328449173521</v>
       </c>
       <c r="D293">
-        <v>139.54096420142352</v>
+        <v>137.73534153560257</v>
       </c>
     </row>
     <row r="294" spans="2:4">
@@ -12044,10 +12047,10 @@
         <v>688</v>
       </c>
       <c r="C294">
-        <v>34.205328449173521</v>
+        <v>33.580800418809254</v>
       </c>
       <c r="D294">
-        <v>137.73534153560257</v>
+        <v>139.54096420142346</v>
       </c>
     </row>
     <row r="295" spans="2:4">
@@ -12100,7 +12103,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{871C57FC-F5E9-4CB8-95D0-821140FB08C5}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9A5702C8-DD3E-4FC6-A484-440067E00DEC}">
   <dimension ref="B9:H298"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -15789,7 +15792,7 @@
         <v>693</v>
       </c>
       <c r="H193" t="s">
-        <v>734</v>
+        <v>722</v>
       </c>
     </row>
     <row r="194" spans="2:8">
@@ -15809,7 +15812,7 @@
         <v>693</v>
       </c>
       <c r="H194" t="s">
-        <v>738</v>
+        <v>722</v>
       </c>
     </row>
     <row r="195" spans="2:8">
@@ -15829,7 +15832,7 @@
         <v>693</v>
       </c>
       <c r="H195" t="s">
-        <v>737</v>
+        <v>722</v>
       </c>
     </row>
     <row r="196" spans="2:8">
@@ -15889,7 +15892,7 @@
         <v>693</v>
       </c>
       <c r="H198" t="s">
-        <v>737</v>
+        <v>726</v>
       </c>
     </row>
     <row r="199" spans="2:8">
@@ -15909,7 +15912,7 @@
         <v>693</v>
       </c>
       <c r="H199" t="s">
-        <v>737</v>
+        <v>722</v>
       </c>
     </row>
     <row r="200" spans="2:8">
@@ -15929,7 +15932,7 @@
         <v>693</v>
       </c>
       <c r="H200" t="s">
-        <v>737</v>
+        <v>718</v>
       </c>
     </row>
     <row r="201" spans="2:8">
@@ -15949,7 +15952,7 @@
         <v>693</v>
       </c>
       <c r="H201" t="s">
-        <v>737</v>
+        <v>710</v>
       </c>
     </row>
     <row r="202" spans="2:8">
@@ -15969,7 +15972,7 @@
         <v>693</v>
       </c>
       <c r="H202" t="s">
-        <v>722</v>
+        <v>703</v>
       </c>
     </row>
     <row r="203" spans="2:8">
@@ -15989,7 +15992,7 @@
         <v>693</v>
       </c>
       <c r="H203" t="s">
-        <v>722</v>
+        <v>702</v>
       </c>
     </row>
     <row r="204" spans="2:8">
@@ -16009,7 +16012,7 @@
         <v>693</v>
       </c>
       <c r="H204" t="s">
-        <v>726</v>
+        <v>722</v>
       </c>
     </row>
     <row r="205" spans="2:8">
@@ -16029,7 +16032,7 @@
         <v>693</v>
       </c>
       <c r="H205" t="s">
-        <v>703</v>
+        <v>733</v>
       </c>
     </row>
     <row r="206" spans="2:8">
@@ -16049,7 +16052,7 @@
         <v>693</v>
       </c>
       <c r="H206" t="s">
-        <v>700</v>
+        <v>737</v>
       </c>
     </row>
     <row r="207" spans="2:8">
@@ -16069,7 +16072,7 @@
         <v>693</v>
       </c>
       <c r="H207" t="s">
-        <v>722</v>
+        <v>737</v>
       </c>
     </row>
     <row r="208" spans="2:8">
@@ -16089,7 +16092,7 @@
         <v>693</v>
       </c>
       <c r="H208" t="s">
-        <v>718</v>
+        <v>737</v>
       </c>
     </row>
     <row r="209" spans="2:8">
@@ -16109,7 +16112,7 @@
         <v>693</v>
       </c>
       <c r="H209" t="s">
-        <v>730</v>
+        <v>722</v>
       </c>
     </row>
     <row r="210" spans="2:8">
@@ -16129,7 +16132,7 @@
         <v>693</v>
       </c>
       <c r="H210" t="s">
-        <v>733</v>
+        <v>737</v>
       </c>
     </row>
     <row r="211" spans="2:8">
@@ -16149,7 +16152,7 @@
         <v>693</v>
       </c>
       <c r="H211" t="s">
-        <v>722</v>
+        <v>737</v>
       </c>
     </row>
     <row r="212" spans="2:8">
@@ -16169,7 +16172,7 @@
         <v>693</v>
       </c>
       <c r="H212" t="s">
-        <v>739</v>
+        <v>722</v>
       </c>
     </row>
     <row r="213" spans="2:8">
@@ -16229,7 +16232,7 @@
         <v>693</v>
       </c>
       <c r="H215" t="s">
-        <v>722</v>
+        <v>705</v>
       </c>
     </row>
     <row r="216" spans="2:8">
@@ -16249,7 +16252,7 @@
         <v>693</v>
       </c>
       <c r="H216" t="s">
-        <v>722</v>
+        <v>694</v>
       </c>
     </row>
     <row r="217" spans="2:8">
@@ -16269,7 +16272,7 @@
         <v>693</v>
       </c>
       <c r="H217" t="s">
-        <v>705</v>
+        <v>714</v>
       </c>
     </row>
     <row r="218" spans="2:8">
@@ -16289,7 +16292,7 @@
         <v>693</v>
       </c>
       <c r="H218" t="s">
-        <v>694</v>
+        <v>722</v>
       </c>
     </row>
     <row r="219" spans="2:8">
@@ -16309,7 +16312,7 @@
         <v>693</v>
       </c>
       <c r="H219" t="s">
-        <v>720</v>
+        <v>738</v>
       </c>
     </row>
     <row r="220" spans="2:8">
@@ -16329,7 +16332,7 @@
         <v>693</v>
       </c>
       <c r="H220" t="s">
-        <v>699</v>
+        <v>720</v>
       </c>
     </row>
     <row r="221" spans="2:8">
@@ -16349,7 +16352,7 @@
         <v>693</v>
       </c>
       <c r="H221" t="s">
-        <v>722</v>
+        <v>739</v>
       </c>
     </row>
     <row r="222" spans="2:8">
@@ -16369,7 +16372,7 @@
         <v>693</v>
       </c>
       <c r="H222" t="s">
-        <v>722</v>
+        <v>734</v>
       </c>
     </row>
     <row r="223" spans="2:8">
@@ -16389,7 +16392,7 @@
         <v>693</v>
       </c>
       <c r="H223" t="s">
-        <v>714</v>
+        <v>734</v>
       </c>
     </row>
     <row r="224" spans="2:8">
@@ -17089,7 +17092,7 @@
         <v>693</v>
       </c>
       <c r="H258" t="s">
-        <v>739</v>
+        <v>740</v>
       </c>
     </row>
     <row r="259" spans="2:8">
@@ -17309,7 +17312,7 @@
         <v>693</v>
       </c>
       <c r="H269" t="s">
-        <v>737</v>
+        <v>722</v>
       </c>
     </row>
     <row r="270" spans="2:8">
@@ -17329,7 +17332,7 @@
         <v>693</v>
       </c>
       <c r="H270" t="s">
-        <v>722</v>
+        <v>737</v>
       </c>
     </row>
     <row r="271" spans="2:8">
@@ -17409,7 +17412,7 @@
         <v>693</v>
       </c>
       <c r="H274" t="s">
-        <v>722</v>
+        <v>737</v>
       </c>
     </row>
     <row r="275" spans="2:8">

</xml_diff>

<commit_message>
Updated JPN_grids model - 2025-09-22 09:16
</commit_message>
<xml_diff>
--- a/VerveStacks_JPN_grids/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_JPN_grids/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_JPN_grids\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{4AEBD19E-40D1-4F38-AF1C-E80959B29F8D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{575FE622-9F38-4F18-89B0-1A7C966E8126}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -8909,7 +8909,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4BA644FC-647E-460B-886F-4CF924F99980}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E94F2948-6B27-4080-A14D-E85369C74425}">
   <dimension ref="B9:D298"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -12103,7 +12103,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9A5702C8-DD3E-4FC6-A484-440067E00DEC}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{17AC6F4C-6D18-44E7-B545-3049D697CEE0}">
   <dimension ref="B9:H298"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated JPN_grids model - 2025-09-22 10:00
</commit_message>
<xml_diff>
--- a/VerveStacks_JPN_grids/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_JPN_grids/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_JPN_grids\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{575FE622-9F38-4F18-89B0-1A7C966E8126}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{76313C0E-F9D8-4317-ADD4-6594A28F591C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -8909,7 +8909,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E94F2948-6B27-4080-A14D-E85369C74425}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{834A047F-31D6-4640-B35B-9D3CCC058B1A}">
   <dimension ref="B9:D298"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -12103,7 +12103,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{17AC6F4C-6D18-44E7-B545-3049D697CEE0}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3FCA273F-045D-4586-9162-B8579E0F3A2C}">
   <dimension ref="B9:H298"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated JPN_grids model - 2025-09-22 11:26
</commit_message>
<xml_diff>
--- a/VerveStacks_JPN_grids/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_JPN_grids/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_JPN_grids\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{76313C0E-F9D8-4317-ADD4-6594A28F591C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{2F1CE32E-D496-41D0-8300-034F54DA2D6C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -8909,7 +8909,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{834A047F-31D6-4640-B35B-9D3CCC058B1A}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{202E54F5-5230-4C50-9681-2FD5176E15AF}">
   <dimension ref="B9:D298"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -12103,7 +12103,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3FCA273F-045D-4586-9162-B8579E0F3A2C}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8B1F5C36-881B-4B16-9A79-6869C0DD73BD}">
   <dimension ref="B9:H298"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated JPN_grids model - 2025-09-22 11:45
</commit_message>
<xml_diff>
--- a/VerveStacks_JPN_grids/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_JPN_grids/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_JPN_grids\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{2F1CE32E-D496-41D0-8300-034F54DA2D6C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{DBCDC7A7-04DA-44E7-B58F-E6F05C1FBC1C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -8909,7 +8909,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{202E54F5-5230-4C50-9681-2FD5176E15AF}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ADD675D2-AA14-4F01-8AED-06214EB50F5B}">
   <dimension ref="B9:D298"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -12103,7 +12103,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8B1F5C36-881B-4B16-9A79-6869C0DD73BD}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{68B3DEE2-3C1A-454B-AC30-828BFD0ED024}">
   <dimension ref="B9:H298"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated JPN_grids model - 2025-09-22 11:49
</commit_message>
<xml_diff>
--- a/VerveStacks_JPN_grids/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_JPN_grids/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_JPN_grids\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{DBCDC7A7-04DA-44E7-B58F-E6F05C1FBC1C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{056D8C02-35B9-486E-825B-D7B2C4F41F7E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -8909,7 +8909,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ADD675D2-AA14-4F01-8AED-06214EB50F5B}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3EF7FAEB-6820-40D9-B101-BD8B7581CA30}">
   <dimension ref="B9:D298"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -12103,7 +12103,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{68B3DEE2-3C1A-454B-AC30-828BFD0ED024}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CC59C412-4B03-4803-82FA-7A6C3AEB9103}">
   <dimension ref="B9:H298"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated JPN_grids model - 2025-09-22 11:59
</commit_message>
<xml_diff>
--- a/VerveStacks_JPN_grids/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_JPN_grids/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_JPN_grids\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{056D8C02-35B9-486E-825B-D7B2C4F41F7E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{DAD94377-F589-4B1D-9E95-2CD2D3DFF1DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -8909,7 +8909,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3EF7FAEB-6820-40D9-B101-BD8B7581CA30}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{54EC1EBE-18D8-4CA2-A9E7-76ADD807784B}">
   <dimension ref="B9:D298"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -12103,7 +12103,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CC59C412-4B03-4803-82FA-7A6C3AEB9103}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C6119B78-7FDE-457E-9D12-1655FE671368}">
   <dimension ref="B9:H298"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated JPN_grids model - 2025-09-22 13:13
</commit_message>
<xml_diff>
--- a/VerveStacks_JPN_grids/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_JPN_grids/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_JPN_grids\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{DAD94377-F589-4B1D-9E95-2CD2D3DFF1DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{19C99289-F6F0-4345-BEC6-388A707BF84F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -8909,7 +8909,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{54EC1EBE-18D8-4CA2-A9E7-76ADD807784B}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{73DBB423-E931-42EF-B99D-F0737BDA7A74}">
   <dimension ref="B9:D298"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -12103,7 +12103,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C6119B78-7FDE-457E-9D12-1655FE671368}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6C026A83-A83B-4778-AF65-3A2ACC48880E}">
   <dimension ref="B9:H298"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated JPN_grids model - 2025-09-22 14:04
</commit_message>
<xml_diff>
--- a/VerveStacks_JPN_grids/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_JPN_grids/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_JPN_grids\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{19C99289-F6F0-4345-BEC6-388A707BF84F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{2D686C4B-FB33-4B7E-AF70-B329DCA54AB9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -8909,7 +8909,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{73DBB423-E931-42EF-B99D-F0737BDA7A74}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7523F016-93E2-4941-ADD6-49FB5FE9DC04}">
   <dimension ref="B9:D298"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -12103,7 +12103,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6C026A83-A83B-4778-AF65-3A2ACC48880E}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{18EEE888-5AE2-4DCF-9407-E3BE274C768A}">
   <dimension ref="B9:H298"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>